<commit_message>
Enhance account management by adding new SBER accounts for ИП Парфененко, ООО М-Инвест, and others; update display names and company account lists accordingly.
</commit_message>
<xml_diff>
--- a/Расчетные счета.xlsx
+++ b/Расчетные счета.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="222">
   <si>
     <t>Параметры:</t>
   </si>
@@ -154,12 +154,15 @@
     <t>42102810990270017489</t>
   </si>
   <si>
+    <t>40702810200810143018</t>
+  </si>
+  <si>
+    <t>МЕДИА 47 ООО</t>
+  </si>
+  <si>
     <t>40702810755000147485</t>
   </si>
   <si>
-    <t>МЕДИА 47 ООО</t>
-  </si>
-  <si>
     <t>40702810255710014683</t>
   </si>
   <si>
@@ -238,12 +241,15 @@
     <t>42102810255000561677</t>
   </si>
   <si>
+    <t>40702810255710018524</t>
+  </si>
+  <si>
+    <t>ООО "М-ИНВЕСТ"</t>
+  </si>
+  <si>
     <t>40702810920020003209</t>
   </si>
   <si>
-    <t>ООО "М-ИНВЕСТ"</t>
-  </si>
-  <si>
     <t>40702810555710014697</t>
   </si>
   <si>
@@ -581,6 +587,9 @@
   </si>
   <si>
     <t>40702810555710013588</t>
+  </si>
+  <si>
+    <t>40702810900810114318</t>
   </si>
   <si>
     <t>42102810620020036093</t>
@@ -835,7 +844,7 @@
     <outlinePr summaryBelow="false" summaryRight="false"/>
     <pageSetUpPr autoPageBreaks="false" fitToPage="true"/>
   </sheetPr>
-  <dimension ref="H168"/>
+  <dimension ref="H171"/>
   <sheetFormatPr defaultColWidth="10.5" customHeight="true" defaultRowHeight="11.429"/>
   <cols>
     <col min="1" max="1" width="10.5" style="1" customWidth="true"/>
@@ -1382,7 +1391,7 @@
       <c r="E35" s="4" t="e"/>
       <c r="F35" s="4" t="e"/>
       <c r="G35" s="4" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H35" s="5" t="n">
         <v>1</v>
@@ -1395,7 +1404,7 @@
       <c r="B36" s="4" t="e"/>
       <c r="C36" s="4" t="e"/>
       <c r="D36" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E36" s="4" t="e"/>
       <c r="F36" s="4" t="e"/>
@@ -1408,17 +1417,17 @@
     </row>
     <row r="37" ht="25" customHeight="true">
       <c r="A37" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B37" s="4" t="e"/>
       <c r="C37" s="4" t="e"/>
       <c r="D37" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E37" s="4" t="e"/>
       <c r="F37" s="4" t="e"/>
       <c r="G37" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H37" s="5" t="n">
         <v>1</v>
@@ -1431,12 +1440,12 @@
       <c r="B38" s="4" t="e"/>
       <c r="C38" s="4" t="e"/>
       <c r="D38" s="4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E38" s="4" t="e"/>
       <c r="F38" s="4" t="e"/>
       <c r="G38" s="4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="H38" s="5" t="n">
         <v>1</v>
@@ -1444,17 +1453,17 @@
     </row>
     <row r="39" ht="25" customHeight="true">
       <c r="A39" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B39" s="4" t="e"/>
       <c r="C39" s="4" t="e"/>
       <c r="D39" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E39" s="4" t="e"/>
       <c r="F39" s="4" t="e"/>
       <c r="G39" s="4" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H39" s="5" t="n">
         <v>1</v>
@@ -1462,17 +1471,17 @@
     </row>
     <row r="40" ht="25" customHeight="true">
       <c r="A40" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B40" s="4" t="e"/>
       <c r="C40" s="4" t="e"/>
       <c r="D40" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E40" s="4" t="e"/>
       <c r="F40" s="4" t="e"/>
       <c r="G40" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H40" s="5" t="n">
         <v>1</v>
@@ -1485,7 +1494,7 @@
       <c r="B41" s="4" t="e"/>
       <c r="C41" s="4" t="e"/>
       <c r="D41" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E41" s="4" t="e"/>
       <c r="F41" s="4" t="e"/>
@@ -1498,17 +1507,17 @@
     </row>
     <row r="42" ht="25" customHeight="true">
       <c r="A42" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B42" s="4" t="e"/>
       <c r="C42" s="4" t="e"/>
       <c r="D42" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E42" s="4" t="e"/>
       <c r="F42" s="4" t="e"/>
       <c r="G42" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H42" s="5" t="n">
         <v>1</v>
@@ -1521,12 +1530,12 @@
       <c r="B43" s="4" t="e"/>
       <c r="C43" s="4" t="e"/>
       <c r="D43" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E43" s="4" t="e"/>
       <c r="F43" s="4" t="e"/>
       <c r="G43" s="4" t="s">
-        <v>58</v>
+        <v>11</v>
       </c>
       <c r="H43" s="5" t="n">
         <v>1</v>
@@ -1534,17 +1543,17 @@
     </row>
     <row r="44" ht="25" customHeight="true">
       <c r="A44" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B44" s="4" t="e"/>
       <c r="C44" s="4" t="e"/>
       <c r="D44" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E44" s="4" t="e"/>
       <c r="F44" s="4" t="e"/>
       <c r="G44" s="4" t="s">
-        <v>25</v>
+        <v>59</v>
       </c>
       <c r="H44" s="5" t="n">
         <v>1</v>
@@ -1557,12 +1566,12 @@
       <c r="B45" s="4" t="e"/>
       <c r="C45" s="4" t="e"/>
       <c r="D45" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E45" s="4" t="e"/>
       <c r="F45" s="4" t="e"/>
       <c r="G45" s="4" t="s">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="H45" s="5" t="n">
         <v>1</v>
@@ -1575,12 +1584,12 @@
       <c r="B46" s="4" t="e"/>
       <c r="C46" s="4" t="e"/>
       <c r="D46" s="4" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E46" s="4" t="e"/>
       <c r="F46" s="4" t="e"/>
       <c r="G46" s="4" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
       <c r="H46" s="5" t="n">
         <v>1</v>
@@ -1588,17 +1597,17 @@
     </row>
     <row r="47" ht="25" customHeight="true">
       <c r="A47" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B47" s="4" t="e"/>
       <c r="C47" s="4" t="e"/>
       <c r="D47" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E47" s="4" t="e"/>
       <c r="F47" s="4" t="e"/>
       <c r="G47" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H47" s="5" t="n">
         <v>1</v>
@@ -1611,12 +1620,12 @@
       <c r="B48" s="4" t="e"/>
       <c r="C48" s="4" t="e"/>
       <c r="D48" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E48" s="4" t="e"/>
       <c r="F48" s="4" t="e"/>
       <c r="G48" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H48" s="5" t="n">
         <v>1</v>
@@ -1624,17 +1633,17 @@
     </row>
     <row r="49" ht="25" customHeight="true">
       <c r="A49" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B49" s="4" t="e"/>
       <c r="C49" s="4" t="e"/>
       <c r="D49" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E49" s="4" t="e"/>
       <c r="F49" s="4" t="e"/>
       <c r="G49" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H49" s="5" t="n">
         <v>1</v>
@@ -1647,12 +1656,12 @@
       <c r="B50" s="4" t="e"/>
       <c r="C50" s="4" t="e"/>
       <c r="D50" s="4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E50" s="4" t="e"/>
       <c r="F50" s="4" t="e"/>
       <c r="G50" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H50" s="5" t="n">
         <v>1</v>
@@ -1660,12 +1669,12 @@
     </row>
     <row r="51" ht="25" customHeight="true">
       <c r="A51" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B51" s="4" t="e"/>
       <c r="C51" s="4" t="e"/>
       <c r="D51" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E51" s="4" t="e"/>
       <c r="F51" s="4" t="e"/>
@@ -1683,7 +1692,7 @@
       <c r="B52" s="4" t="e"/>
       <c r="C52" s="4" t="e"/>
       <c r="D52" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E52" s="4" t="e"/>
       <c r="F52" s="4" t="e"/>
@@ -1701,12 +1710,12 @@
       <c r="B53" s="4" t="e"/>
       <c r="C53" s="4" t="e"/>
       <c r="D53" s="4" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E53" s="4" t="e"/>
       <c r="F53" s="4" t="e"/>
       <c r="G53" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H53" s="5" t="n">
         <v>1</v>
@@ -1714,12 +1723,12 @@
     </row>
     <row r="54" ht="25" customHeight="true">
       <c r="A54" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B54" s="4" t="e"/>
       <c r="C54" s="4" t="e"/>
       <c r="D54" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E54" s="4" t="e"/>
       <c r="F54" s="4" t="e"/>
@@ -1732,12 +1741,12 @@
     </row>
     <row r="55" ht="25" customHeight="true">
       <c r="A55" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B55" s="4" t="e"/>
       <c r="C55" s="4" t="e"/>
       <c r="D55" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E55" s="4" t="e"/>
       <c r="F55" s="4" t="e"/>
@@ -1750,12 +1759,12 @@
     </row>
     <row r="56" ht="25" customHeight="true">
       <c r="A56" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B56" s="4" t="e"/>
       <c r="C56" s="4" t="e"/>
       <c r="D56" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E56" s="4" t="e"/>
       <c r="F56" s="4" t="e"/>
@@ -1768,17 +1777,17 @@
     </row>
     <row r="57" ht="25" customHeight="true">
       <c r="A57" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B57" s="4" t="e"/>
       <c r="C57" s="4" t="e"/>
       <c r="D57" s="4" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E57" s="4" t="e"/>
       <c r="F57" s="4" t="e"/>
       <c r="G57" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H57" s="5" t="n">
         <v>1</v>
@@ -1786,7 +1795,7 @@
     </row>
     <row r="58" ht="25" customHeight="true">
       <c r="A58" s="4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B58" s="4" t="e"/>
       <c r="C58" s="4" t="e"/>
@@ -1796,7 +1805,7 @@
       <c r="E58" s="4" t="e"/>
       <c r="F58" s="4" t="e"/>
       <c r="G58" s="4" t="s">
-        <v>81</v>
+        <v>11</v>
       </c>
       <c r="H58" s="5" t="n">
         <v>1</v>
@@ -1804,17 +1813,17 @@
     </row>
     <row r="59" ht="25" customHeight="true">
       <c r="A59" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B59" s="4" t="e"/>
       <c r="C59" s="4" t="e"/>
       <c r="D59" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E59" s="4" t="e"/>
       <c r="F59" s="4" t="e"/>
       <c r="G59" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="H59" s="5" t="n">
         <v>1</v>
@@ -1822,17 +1831,17 @@
     </row>
     <row r="60" ht="25" customHeight="true">
       <c r="A60" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B60" s="4" t="e"/>
       <c r="C60" s="4" t="e"/>
       <c r="D60" s="4" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E60" s="4" t="e"/>
       <c r="F60" s="4" t="e"/>
       <c r="G60" s="4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="H60" s="5" t="n">
         <v>1</v>
@@ -1840,7 +1849,7 @@
     </row>
     <row r="61" ht="25" customHeight="true">
       <c r="A61" s="4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B61" s="4" t="e"/>
       <c r="C61" s="4" t="e"/>
@@ -1850,7 +1859,7 @@
       <c r="E61" s="4" t="e"/>
       <c r="F61" s="4" t="e"/>
       <c r="G61" s="4" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="H61" s="5" t="n">
         <v>1</v>
@@ -1858,17 +1867,17 @@
     </row>
     <row r="62" ht="25" customHeight="true">
       <c r="A62" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B62" s="4" t="e"/>
       <c r="C62" s="4" t="e"/>
       <c r="D62" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E62" s="4" t="e"/>
       <c r="F62" s="4" t="e"/>
       <c r="G62" s="4" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="H62" s="5" t="n">
         <v>1</v>
@@ -1881,15 +1890,15 @@
       <c r="B63" s="4" t="e"/>
       <c r="C63" s="4" t="e"/>
       <c r="D63" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E63" s="4" t="e"/>
       <c r="F63" s="4" t="e"/>
       <c r="G63" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" ht="25" customHeight="true">
@@ -1899,12 +1908,12 @@
       <c r="B64" s="4" t="e"/>
       <c r="C64" s="4" t="e"/>
       <c r="D64" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E64" s="4" t="e"/>
       <c r="F64" s="4" t="e"/>
       <c r="G64" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H64" s="5" t="n">
         <v>1</v>
@@ -1917,7 +1926,7 @@
       <c r="B65" s="4" t="e"/>
       <c r="C65" s="4" t="e"/>
       <c r="D65" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E65" s="4" t="e"/>
       <c r="F65" s="4" t="e"/>
@@ -1925,7 +1934,7 @@
         <v>13</v>
       </c>
       <c r="H65" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66" ht="25" customHeight="true">
@@ -1935,7 +1944,7 @@
       <c r="B66" s="4" t="e"/>
       <c r="C66" s="4" t="e"/>
       <c r="D66" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E66" s="4" t="e"/>
       <c r="F66" s="4" t="e"/>
@@ -1953,7 +1962,7 @@
       <c r="B67" s="4" t="e"/>
       <c r="C67" s="4" t="e"/>
       <c r="D67" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E67" s="4" t="e"/>
       <c r="F67" s="4" t="e"/>
@@ -1971,7 +1980,7 @@
       <c r="B68" s="4" t="e"/>
       <c r="C68" s="4" t="e"/>
       <c r="D68" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E68" s="4" t="e"/>
       <c r="F68" s="4" t="e"/>
@@ -1989,7 +1998,7 @@
       <c r="B69" s="4" t="e"/>
       <c r="C69" s="4" t="e"/>
       <c r="D69" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E69" s="4" t="e"/>
       <c r="F69" s="4" t="e"/>
@@ -2007,7 +2016,7 @@
       <c r="B70" s="4" t="e"/>
       <c r="C70" s="4" t="e"/>
       <c r="D70" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E70" s="4" t="e"/>
       <c r="F70" s="4" t="e"/>
@@ -2025,7 +2034,7 @@
       <c r="B71" s="4" t="e"/>
       <c r="C71" s="4" t="e"/>
       <c r="D71" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E71" s="4" t="e"/>
       <c r="F71" s="4" t="e"/>
@@ -2043,7 +2052,7 @@
       <c r="B72" s="4" t="e"/>
       <c r="C72" s="4" t="e"/>
       <c r="D72" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E72" s="4" t="e"/>
       <c r="F72" s="4" t="e"/>
@@ -2061,7 +2070,7 @@
       <c r="B73" s="4" t="e"/>
       <c r="C73" s="4" t="e"/>
       <c r="D73" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E73" s="4" t="e"/>
       <c r="F73" s="4" t="e"/>
@@ -2079,7 +2088,7 @@
       <c r="B74" s="4" t="e"/>
       <c r="C74" s="4" t="e"/>
       <c r="D74" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E74" s="4" t="e"/>
       <c r="F74" s="4" t="e"/>
@@ -2097,7 +2106,7 @@
       <c r="B75" s="4" t="e"/>
       <c r="C75" s="4" t="e"/>
       <c r="D75" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E75" s="4" t="e"/>
       <c r="F75" s="4" t="e"/>
@@ -2115,12 +2124,12 @@
       <c r="B76" s="4" t="e"/>
       <c r="C76" s="4" t="e"/>
       <c r="D76" s="4" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E76" s="4" t="e"/>
       <c r="F76" s="4" t="e"/>
       <c r="G76" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H76" s="5" t="n">
         <v>1</v>
@@ -2128,17 +2137,17 @@
     </row>
     <row r="77" ht="25" customHeight="true">
       <c r="A77" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B77" s="4" t="e"/>
       <c r="C77" s="4" t="e"/>
       <c r="D77" s="4" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E77" s="4" t="e"/>
       <c r="F77" s="4" t="e"/>
       <c r="G77" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H77" s="5" t="n">
         <v>1</v>
@@ -2146,17 +2155,17 @@
     </row>
     <row r="78" ht="25" customHeight="true">
       <c r="A78" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B78" s="4" t="e"/>
       <c r="C78" s="4" t="e"/>
       <c r="D78" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E78" s="4" t="e"/>
       <c r="F78" s="4" t="e"/>
       <c r="G78" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H78" s="5" t="n">
         <v>1</v>
@@ -2169,12 +2178,12 @@
       <c r="B79" s="4" t="e"/>
       <c r="C79" s="4" t="e"/>
       <c r="D79" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E79" s="4" t="e"/>
       <c r="F79" s="4" t="e"/>
       <c r="G79" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H79" s="5" t="n">
         <v>1</v>
@@ -2187,7 +2196,7 @@
       <c r="B80" s="4" t="e"/>
       <c r="C80" s="4" t="e"/>
       <c r="D80" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E80" s="4" t="e"/>
       <c r="F80" s="4" t="e"/>
@@ -2205,7 +2214,7 @@
       <c r="B81" s="4" t="e"/>
       <c r="C81" s="4" t="e"/>
       <c r="D81" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E81" s="4" t="e"/>
       <c r="F81" s="4" t="e"/>
@@ -2223,7 +2232,7 @@
       <c r="B82" s="4" t="e"/>
       <c r="C82" s="4" t="e"/>
       <c r="D82" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E82" s="4" t="e"/>
       <c r="F82" s="4" t="e"/>
@@ -2241,7 +2250,7 @@
       <c r="B83" s="4" t="e"/>
       <c r="C83" s="4" t="e"/>
       <c r="D83" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E83" s="4" t="e"/>
       <c r="F83" s="4" t="e"/>
@@ -2259,7 +2268,7 @@
       <c r="B84" s="4" t="e"/>
       <c r="C84" s="4" t="e"/>
       <c r="D84" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E84" s="4" t="e"/>
       <c r="F84" s="4" t="e"/>
@@ -2277,7 +2286,7 @@
       <c r="B85" s="4" t="e"/>
       <c r="C85" s="4" t="e"/>
       <c r="D85" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E85" s="4" t="e"/>
       <c r="F85" s="4" t="e"/>
@@ -2295,7 +2304,7 @@
       <c r="B86" s="4" t="e"/>
       <c r="C86" s="4" t="e"/>
       <c r="D86" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E86" s="4" t="e"/>
       <c r="F86" s="4" t="e"/>
@@ -2313,7 +2322,7 @@
       <c r="B87" s="4" t="e"/>
       <c r="C87" s="4" t="e"/>
       <c r="D87" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E87" s="4" t="e"/>
       <c r="F87" s="4" t="e"/>
@@ -2331,7 +2340,7 @@
       <c r="B88" s="4" t="e"/>
       <c r="C88" s="4" t="e"/>
       <c r="D88" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E88" s="4" t="e"/>
       <c r="F88" s="4" t="e"/>
@@ -2349,7 +2358,7 @@
       <c r="B89" s="4" t="e"/>
       <c r="C89" s="4" t="e"/>
       <c r="D89" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E89" s="4" t="e"/>
       <c r="F89" s="4" t="e"/>
@@ -2367,7 +2376,7 @@
       <c r="B90" s="4" t="e"/>
       <c r="C90" s="4" t="e"/>
       <c r="D90" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E90" s="4" t="e"/>
       <c r="F90" s="4" t="e"/>
@@ -2385,7 +2394,7 @@
       <c r="B91" s="4" t="e"/>
       <c r="C91" s="4" t="e"/>
       <c r="D91" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E91" s="4" t="e"/>
       <c r="F91" s="4" t="e"/>
@@ -2403,7 +2412,7 @@
       <c r="B92" s="4" t="e"/>
       <c r="C92" s="4" t="e"/>
       <c r="D92" s="4" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="E92" s="4" t="e"/>
       <c r="F92" s="4" t="e"/>
@@ -2416,17 +2425,17 @@
     </row>
     <row r="93" ht="25" customHeight="true">
       <c r="A93" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B93" s="4" t="e"/>
       <c r="C93" s="4" t="e"/>
       <c r="D93" s="4" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="E93" s="4" t="e"/>
       <c r="F93" s="4" t="e"/>
       <c r="G93" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H93" s="5" t="n">
         <v>1</v>
@@ -2434,17 +2443,17 @@
     </row>
     <row r="94" ht="25" customHeight="true">
       <c r="A94" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B94" s="4" t="e"/>
       <c r="C94" s="4" t="e"/>
       <c r="D94" s="4" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E94" s="4" t="e"/>
       <c r="F94" s="4" t="e"/>
       <c r="G94" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H94" s="5" t="n">
         <v>1</v>
@@ -2457,12 +2466,12 @@
       <c r="B95" s="4" t="e"/>
       <c r="C95" s="4" t="e"/>
       <c r="D95" s="4" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E95" s="4" t="e"/>
       <c r="F95" s="4" t="e"/>
       <c r="G95" s="4" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="H95" s="5" t="n">
         <v>1</v>
@@ -2470,12 +2479,12 @@
     </row>
     <row r="96" ht="25" customHeight="true">
       <c r="A96" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B96" s="4" t="e"/>
       <c r="C96" s="4" t="e"/>
       <c r="D96" s="4" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E96" s="4" t="e"/>
       <c r="F96" s="4" t="e"/>
@@ -2488,7 +2497,7 @@
     </row>
     <row r="97" ht="25" customHeight="true">
       <c r="A97" s="4" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B97" s="4" t="e"/>
       <c r="C97" s="4" t="e"/>
@@ -2498,7 +2507,7 @@
       <c r="E97" s="4" t="e"/>
       <c r="F97" s="4" t="e"/>
       <c r="G97" s="4" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H97" s="5" t="n">
         <v>1</v>
@@ -2506,17 +2515,17 @@
     </row>
     <row r="98" ht="25" customHeight="true">
       <c r="A98" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B98" s="4" t="e"/>
       <c r="C98" s="4" t="e"/>
       <c r="D98" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E98" s="4" t="e"/>
       <c r="F98" s="4" t="e"/>
       <c r="G98" s="4" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H98" s="5" t="n">
         <v>1</v>
@@ -2529,7 +2538,7 @@
       <c r="B99" s="4" t="e"/>
       <c r="C99" s="4" t="e"/>
       <c r="D99" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E99" s="4" t="e"/>
       <c r="F99" s="4" t="e"/>
@@ -2547,7 +2556,7 @@
       <c r="B100" s="4" t="e"/>
       <c r="C100" s="4" t="e"/>
       <c r="D100" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E100" s="4" t="e"/>
       <c r="F100" s="4" t="e"/>
@@ -2565,7 +2574,7 @@
       <c r="B101" s="4" t="e"/>
       <c r="C101" s="4" t="e"/>
       <c r="D101" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E101" s="4" t="e"/>
       <c r="F101" s="4" t="e"/>
@@ -2583,7 +2592,7 @@
       <c r="B102" s="4" t="e"/>
       <c r="C102" s="4" t="e"/>
       <c r="D102" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E102" s="4" t="e"/>
       <c r="F102" s="4" t="e"/>
@@ -2601,7 +2610,7 @@
       <c r="B103" s="4" t="e"/>
       <c r="C103" s="4" t="e"/>
       <c r="D103" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E103" s="4" t="e"/>
       <c r="F103" s="4" t="e"/>
@@ -2619,7 +2628,7 @@
       <c r="B104" s="4" t="e"/>
       <c r="C104" s="4" t="e"/>
       <c r="D104" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E104" s="4" t="e"/>
       <c r="F104" s="4" t="e"/>
@@ -2637,7 +2646,7 @@
       <c r="B105" s="4" t="e"/>
       <c r="C105" s="4" t="e"/>
       <c r="D105" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E105" s="4" t="e"/>
       <c r="F105" s="4" t="e"/>
@@ -2655,7 +2664,7 @@
       <c r="B106" s="4" t="e"/>
       <c r="C106" s="4" t="e"/>
       <c r="D106" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E106" s="4" t="e"/>
       <c r="F106" s="4" t="e"/>
@@ -2673,7 +2682,7 @@
       <c r="B107" s="4" t="e"/>
       <c r="C107" s="4" t="e"/>
       <c r="D107" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E107" s="4" t="e"/>
       <c r="F107" s="4" t="e"/>
@@ -2691,7 +2700,7 @@
       <c r="B108" s="4" t="e"/>
       <c r="C108" s="4" t="e"/>
       <c r="D108" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E108" s="4" t="e"/>
       <c r="F108" s="4" t="e"/>
@@ -2709,7 +2718,7 @@
       <c r="B109" s="4" t="e"/>
       <c r="C109" s="4" t="e"/>
       <c r="D109" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E109" s="4" t="e"/>
       <c r="F109" s="4" t="e"/>
@@ -2727,7 +2736,7 @@
       <c r="B110" s="4" t="e"/>
       <c r="C110" s="4" t="e"/>
       <c r="D110" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E110" s="4" t="e"/>
       <c r="F110" s="4" t="e"/>
@@ -2745,7 +2754,7 @@
       <c r="B111" s="4" t="e"/>
       <c r="C111" s="4" t="e"/>
       <c r="D111" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E111" s="4" t="e"/>
       <c r="F111" s="4" t="e"/>
@@ -2763,7 +2772,7 @@
       <c r="B112" s="4" t="e"/>
       <c r="C112" s="4" t="e"/>
       <c r="D112" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E112" s="4" t="e"/>
       <c r="F112" s="4" t="e"/>
@@ -2781,12 +2790,12 @@
       <c r="B113" s="4" t="e"/>
       <c r="C113" s="4" t="e"/>
       <c r="D113" s="4" t="s">
-        <v>144</v>
+        <v>128</v>
       </c>
       <c r="E113" s="4" t="e"/>
       <c r="F113" s="4" t="e"/>
       <c r="G113" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="H113" s="5" t="n">
         <v>1</v>
@@ -2794,12 +2803,12 @@
     </row>
     <row r="114" ht="25" customHeight="true">
       <c r="A114" s="4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B114" s="4" t="e"/>
       <c r="C114" s="4" t="e"/>
       <c r="D114" s="4" t="s">
-        <v>144</v>
+        <v>128</v>
       </c>
       <c r="E114" s="4" t="e"/>
       <c r="F114" s="4" t="e"/>
@@ -2812,12 +2821,12 @@
     </row>
     <row r="115" ht="25" customHeight="true">
       <c r="A115" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B115" s="4" t="e"/>
       <c r="C115" s="4" t="e"/>
       <c r="D115" s="4" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E115" s="4" t="e"/>
       <c r="F115" s="4" t="e"/>
@@ -2835,12 +2844,12 @@
       <c r="B116" s="4" t="e"/>
       <c r="C116" s="4" t="e"/>
       <c r="D116" s="4" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E116" s="4" t="e"/>
       <c r="F116" s="4" t="e"/>
       <c r="G116" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="H116" s="5" t="n">
         <v>1</v>
@@ -2853,12 +2862,12 @@
       <c r="B117" s="4" t="e"/>
       <c r="C117" s="4" t="e"/>
       <c r="D117" s="4" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E117" s="4" t="e"/>
       <c r="F117" s="4" t="e"/>
       <c r="G117" s="4" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="H117" s="5" t="n">
         <v>1</v>
@@ -2866,17 +2875,17 @@
     </row>
     <row r="118" ht="25" customHeight="true">
       <c r="A118" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B118" s="4" t="e"/>
       <c r="C118" s="4" t="e"/>
       <c r="D118" s="4" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E118" s="4" t="e"/>
       <c r="F118" s="4" t="e"/>
       <c r="G118" s="4" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="H118" s="5" t="n">
         <v>1</v>
@@ -2884,17 +2893,17 @@
     </row>
     <row r="119" ht="25" customHeight="true">
       <c r="A119" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B119" s="4" t="e"/>
       <c r="C119" s="4" t="e"/>
       <c r="D119" s="4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E119" s="4" t="e"/>
       <c r="F119" s="4" t="e"/>
       <c r="G119" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H119" s="5" t="n">
         <v>1</v>
@@ -2907,12 +2916,12 @@
       <c r="B120" s="4" t="e"/>
       <c r="C120" s="4" t="e"/>
       <c r="D120" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E120" s="4" t="e"/>
       <c r="F120" s="4" t="e"/>
       <c r="G120" s="4" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="H120" s="5" t="n">
         <v>1</v>
@@ -2920,17 +2929,17 @@
     </row>
     <row r="121" ht="25" customHeight="true">
       <c r="A121" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B121" s="4" t="e"/>
       <c r="C121" s="4" t="e"/>
       <c r="D121" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E121" s="4" t="e"/>
       <c r="F121" s="4" t="e"/>
       <c r="G121" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H121" s="5" t="n">
         <v>1</v>
@@ -2938,17 +2947,17 @@
     </row>
     <row r="122" ht="25" customHeight="true">
       <c r="A122" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B122" s="4" t="e"/>
       <c r="C122" s="4" t="e"/>
       <c r="D122" s="4" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E122" s="4" t="e"/>
       <c r="F122" s="4" t="e"/>
       <c r="G122" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H122" s="5" t="n">
         <v>1</v>
@@ -2961,12 +2970,12 @@
       <c r="B123" s="4" t="e"/>
       <c r="C123" s="4" t="e"/>
       <c r="D123" s="4" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E123" s="4" t="e"/>
       <c r="F123" s="4" t="e"/>
       <c r="G123" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="H123" s="5" t="n">
         <v>1</v>
@@ -2979,7 +2988,7 @@
       <c r="B124" s="4" t="e"/>
       <c r="C124" s="4" t="e"/>
       <c r="D124" s="4" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E124" s="4" t="e"/>
       <c r="F124" s="4" t="e"/>
@@ -2987,22 +2996,22 @@
         <v>13</v>
       </c>
       <c r="H124" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="125" ht="25" customHeight="true">
       <c r="A125" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B125" s="4" t="e"/>
       <c r="C125" s="4" t="e"/>
       <c r="D125" s="4" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E125" s="4" t="e"/>
       <c r="F125" s="4" t="e"/>
       <c r="G125" s="4" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="H125" s="5" t="n">
         <v>1</v>
@@ -3010,35 +3019,35 @@
     </row>
     <row r="126" ht="25" customHeight="true">
       <c r="A126" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B126" s="4" t="e"/>
       <c r="C126" s="4" t="e"/>
       <c r="D126" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E126" s="4" t="e"/>
       <c r="F126" s="4" t="e"/>
       <c r="G126" s="4" t="s">
-        <v>162</v>
+        <v>13</v>
       </c>
       <c r="H126" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="127" ht="25" customHeight="true">
       <c r="A127" s="4" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B127" s="4" t="e"/>
       <c r="C127" s="4" t="e"/>
       <c r="D127" s="4" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="E127" s="4" t="e"/>
       <c r="F127" s="4" t="e"/>
       <c r="G127" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H127" s="5" t="n">
         <v>1</v>
@@ -3046,17 +3055,17 @@
     </row>
     <row r="128" ht="25" customHeight="true">
       <c r="A128" s="4" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B128" s="4" t="e"/>
       <c r="C128" s="4" t="e"/>
       <c r="D128" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E128" s="4" t="e"/>
       <c r="F128" s="4" t="e"/>
       <c r="G128" s="4" t="s">
-        <v>11</v>
+        <v>164</v>
       </c>
       <c r="H128" s="5" t="n">
         <v>1</v>
@@ -3064,17 +3073,17 @@
     </row>
     <row r="129" ht="25" customHeight="true">
       <c r="A129" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B129" s="4" t="e"/>
       <c r="C129" s="4" t="e"/>
       <c r="D129" s="4" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E129" s="4" t="e"/>
       <c r="F129" s="4" t="e"/>
       <c r="G129" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H129" s="5" t="n">
         <v>1</v>
@@ -3087,12 +3096,12 @@
       <c r="B130" s="4" t="e"/>
       <c r="C130" s="4" t="e"/>
       <c r="D130" s="4" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E130" s="4" t="e"/>
       <c r="F130" s="4" t="e"/>
       <c r="G130" s="4" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="H130" s="5" t="n">
         <v>1</v>
@@ -3100,17 +3109,17 @@
     </row>
     <row r="131" ht="25" customHeight="true">
       <c r="A131" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B131" s="4" t="e"/>
       <c r="C131" s="4" t="e"/>
       <c r="D131" s="4" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E131" s="4" t="e"/>
       <c r="F131" s="4" t="e"/>
       <c r="G131" s="4" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H131" s="5" t="n">
         <v>1</v>
@@ -3118,17 +3127,17 @@
     </row>
     <row r="132" ht="25" customHeight="true">
       <c r="A132" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B132" s="4" t="e"/>
       <c r="C132" s="4" t="e"/>
       <c r="D132" s="4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="E132" s="4" t="e"/>
       <c r="F132" s="4" t="e"/>
       <c r="G132" s="4" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="H132" s="5" t="n">
         <v>1</v>
@@ -3141,12 +3150,12 @@
       <c r="B133" s="4" t="e"/>
       <c r="C133" s="4" t="e"/>
       <c r="D133" s="4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="E133" s="4" t="e"/>
       <c r="F133" s="4" t="e"/>
       <c r="G133" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="H133" s="5" t="n">
         <v>1</v>
@@ -3159,7 +3168,7 @@
       <c r="B134" s="4" t="e"/>
       <c r="C134" s="4" t="e"/>
       <c r="D134" s="4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="E134" s="4" t="e"/>
       <c r="F134" s="4" t="e"/>
@@ -3177,7 +3186,7 @@
       <c r="B135" s="4" t="e"/>
       <c r="C135" s="4" t="e"/>
       <c r="D135" s="4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="E135" s="4" t="e"/>
       <c r="F135" s="4" t="e"/>
@@ -3195,7 +3204,7 @@
       <c r="B136" s="4" t="e"/>
       <c r="C136" s="4" t="e"/>
       <c r="D136" s="4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="E136" s="4" t="e"/>
       <c r="F136" s="4" t="e"/>
@@ -3213,7 +3222,7 @@
       <c r="B137" s="4" t="e"/>
       <c r="C137" s="4" t="e"/>
       <c r="D137" s="4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="E137" s="4" t="e"/>
       <c r="F137" s="4" t="e"/>
@@ -3231,7 +3240,7 @@
       <c r="B138" s="4" t="e"/>
       <c r="C138" s="4" t="e"/>
       <c r="D138" s="4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="E138" s="4" t="e"/>
       <c r="F138" s="4" t="e"/>
@@ -3249,12 +3258,12 @@
       <c r="B139" s="4" t="e"/>
       <c r="C139" s="4" t="e"/>
       <c r="D139" s="4" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="E139" s="4" t="e"/>
       <c r="F139" s="4" t="e"/>
       <c r="G139" s="4" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="H139" s="5" t="n">
         <v>1</v>
@@ -3262,17 +3271,17 @@
     </row>
     <row r="140" ht="25" customHeight="true">
       <c r="A140" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B140" s="4" t="e"/>
       <c r="C140" s="4" t="e"/>
       <c r="D140" s="4" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="E140" s="4" t="e"/>
       <c r="F140" s="4" t="e"/>
       <c r="G140" s="4" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="H140" s="5" t="n">
         <v>1</v>
@@ -3280,12 +3289,12 @@
     </row>
     <row r="141" ht="25" customHeight="true">
       <c r="A141" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B141" s="4" t="e"/>
       <c r="C141" s="4" t="e"/>
       <c r="D141" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E141" s="4" t="e"/>
       <c r="F141" s="4" t="e"/>
@@ -3298,12 +3307,12 @@
     </row>
     <row r="142" ht="25" customHeight="true">
       <c r="A142" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B142" s="4" t="e"/>
       <c r="C142" s="4" t="e"/>
       <c r="D142" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E142" s="4" t="e"/>
       <c r="F142" s="4" t="e"/>
@@ -3316,17 +3325,17 @@
     </row>
     <row r="143" ht="25" customHeight="true">
       <c r="A143" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B143" s="4" t="e"/>
       <c r="C143" s="4" t="e"/>
       <c r="D143" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E143" s="4" t="e"/>
       <c r="F143" s="4" t="e"/>
       <c r="G143" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H143" s="5" t="n">
         <v>1</v>
@@ -3334,17 +3343,17 @@
     </row>
     <row r="144" ht="25" customHeight="true">
       <c r="A144" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B144" s="4" t="e"/>
       <c r="C144" s="4" t="e"/>
       <c r="D144" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E144" s="4" t="e"/>
       <c r="F144" s="4" t="e"/>
       <c r="G144" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H144" s="5" t="n">
         <v>1</v>
@@ -3352,12 +3361,12 @@
     </row>
     <row r="145" ht="25" customHeight="true">
       <c r="A145" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B145" s="4" t="e"/>
       <c r="C145" s="4" t="e"/>
       <c r="D145" s="4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E145" s="4" t="e"/>
       <c r="F145" s="4" t="e"/>
@@ -3375,12 +3384,12 @@
       <c r="B146" s="4" t="e"/>
       <c r="C146" s="4" t="e"/>
       <c r="D146" s="4" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="E146" s="4" t="e"/>
       <c r="F146" s="4" t="e"/>
       <c r="G146" s="4" t="s">
-        <v>162</v>
+        <v>11</v>
       </c>
       <c r="H146" s="5" t="n">
         <v>1</v>
@@ -3388,17 +3397,17 @@
     </row>
     <row r="147" ht="25" customHeight="true">
       <c r="A147" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B147" s="4" t="e"/>
       <c r="C147" s="4" t="e"/>
       <c r="D147" s="4" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="E147" s="4" t="e"/>
       <c r="F147" s="4" t="e"/>
       <c r="G147" s="4" t="s">
-        <v>162</v>
+        <v>15</v>
       </c>
       <c r="H147" s="5" t="n">
         <v>1</v>
@@ -3406,12 +3415,12 @@
     </row>
     <row r="148" ht="25" customHeight="true">
       <c r="A148" s="4" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B148" s="4" t="e"/>
       <c r="C148" s="4" t="e"/>
       <c r="D148" s="4" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="E148" s="4" t="e"/>
       <c r="F148" s="4" t="e"/>
@@ -3424,17 +3433,17 @@
     </row>
     <row r="149" ht="25" customHeight="true">
       <c r="A149" s="4" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B149" s="4" t="e"/>
       <c r="C149" s="4" t="e"/>
       <c r="D149" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E149" s="4" t="e"/>
       <c r="F149" s="4" t="e"/>
       <c r="G149" s="4" t="s">
-        <v>11</v>
+        <v>164</v>
       </c>
       <c r="H149" s="5" t="n">
         <v>1</v>
@@ -3442,17 +3451,17 @@
     </row>
     <row r="150" ht="25" customHeight="true">
       <c r="A150" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B150" s="4" t="e"/>
       <c r="C150" s="4" t="e"/>
       <c r="D150" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E150" s="4" t="e"/>
       <c r="F150" s="4" t="e"/>
       <c r="G150" s="4" t="s">
-        <v>15</v>
+        <v>164</v>
       </c>
       <c r="H150" s="5" t="n">
         <v>1</v>
@@ -3460,12 +3469,12 @@
     </row>
     <row r="151" ht="25" customHeight="true">
       <c r="A151" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B151" s="4" t="e"/>
       <c r="C151" s="4" t="e"/>
       <c r="D151" s="4" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E151" s="4" t="e"/>
       <c r="F151" s="4" t="e"/>
@@ -3483,12 +3492,12 @@
       <c r="B152" s="4" t="e"/>
       <c r="C152" s="4" t="e"/>
       <c r="D152" s="4" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E152" s="4" t="e"/>
       <c r="F152" s="4" t="e"/>
       <c r="G152" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H152" s="5" t="n">
         <v>1</v>
@@ -3501,12 +3510,12 @@
       <c r="B153" s="4" t="e"/>
       <c r="C153" s="4" t="e"/>
       <c r="D153" s="4" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E153" s="4" t="e"/>
       <c r="F153" s="4" t="e"/>
       <c r="G153" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H153" s="5" t="n">
         <v>1</v>
@@ -3519,7 +3528,7 @@
       <c r="B154" s="4" t="e"/>
       <c r="C154" s="4" t="e"/>
       <c r="D154" s="4" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E154" s="4" t="e"/>
       <c r="F154" s="4" t="e"/>
@@ -3537,7 +3546,7 @@
       <c r="B155" s="4" t="e"/>
       <c r="C155" s="4" t="e"/>
       <c r="D155" s="4" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E155" s="4" t="e"/>
       <c r="F155" s="4" t="e"/>
@@ -3555,7 +3564,7 @@
       <c r="B156" s="4" t="e"/>
       <c r="C156" s="4" t="e"/>
       <c r="D156" s="4" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E156" s="4" t="e"/>
       <c r="F156" s="4" t="e"/>
@@ -3573,7 +3582,7 @@
       <c r="B157" s="4" t="e"/>
       <c r="C157" s="4" t="e"/>
       <c r="D157" s="4" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E157" s="4" t="e"/>
       <c r="F157" s="4" t="e"/>
@@ -3591,7 +3600,7 @@
       <c r="B158" s="4" t="e"/>
       <c r="C158" s="4" t="e"/>
       <c r="D158" s="4" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="E158" s="4" t="e"/>
       <c r="F158" s="4" t="e"/>
@@ -3604,17 +3613,17 @@
     </row>
     <row r="159" ht="25" customHeight="true">
       <c r="A159" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B159" s="4" t="e"/>
       <c r="C159" s="4" t="e"/>
       <c r="D159" s="4" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="E159" s="4" t="e"/>
       <c r="F159" s="4" t="e"/>
       <c r="G159" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H159" s="5" t="n">
         <v>1</v>
@@ -3622,12 +3631,12 @@
     </row>
     <row r="160" ht="25" customHeight="true">
       <c r="A160" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B160" s="4" t="e"/>
       <c r="C160" s="4" t="e"/>
       <c r="D160" s="4" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="E160" s="4" t="e"/>
       <c r="F160" s="4" t="e"/>
@@ -3640,7 +3649,7 @@
     </row>
     <row r="161" ht="25" customHeight="true">
       <c r="A161" s="4" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B161" s="4" t="e"/>
       <c r="C161" s="4" t="e"/>
@@ -3650,7 +3659,7 @@
       <c r="E161" s="4" t="e"/>
       <c r="F161" s="4" t="e"/>
       <c r="G161" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H161" s="5" t="n">
         <v>1</v>
@@ -3658,17 +3667,17 @@
     </row>
     <row r="162" ht="25" customHeight="true">
       <c r="A162" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B162" s="4" t="e"/>
       <c r="C162" s="4" t="e"/>
       <c r="D162" s="4" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="E162" s="4" t="e"/>
       <c r="F162" s="4" t="e"/>
       <c r="G162" s="4" t="s">
-        <v>162</v>
+        <v>11</v>
       </c>
       <c r="H162" s="5" t="n">
         <v>1</v>
@@ -3676,17 +3685,17 @@
     </row>
     <row r="163" ht="25" customHeight="true">
       <c r="A163" s="4" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B163" s="4" t="e"/>
       <c r="C163" s="4" t="e"/>
       <c r="D163" s="4" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="E163" s="4" t="e"/>
       <c r="F163" s="4" t="e"/>
       <c r="G163" s="4" t="s">
-        <v>58</v>
+        <v>13</v>
       </c>
       <c r="H163" s="5" t="n">
         <v>1</v>
@@ -3694,17 +3703,17 @@
     </row>
     <row r="164" ht="25" customHeight="true">
       <c r="A164" s="4" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B164" s="4" t="e"/>
       <c r="C164" s="4" t="e"/>
       <c r="D164" s="4" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="E164" s="4" t="e"/>
       <c r="F164" s="4" t="e"/>
       <c r="G164" s="4" t="s">
-        <v>58</v>
+        <v>11</v>
       </c>
       <c r="H164" s="5" t="n">
         <v>1</v>
@@ -3712,17 +3721,17 @@
     </row>
     <row r="165" ht="25" customHeight="true">
       <c r="A165" s="4" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B165" s="4" t="e"/>
       <c r="C165" s="4" t="e"/>
       <c r="D165" s="4" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E165" s="4" t="e"/>
       <c r="F165" s="4" t="e"/>
       <c r="G165" s="4" t="s">
-        <v>216</v>
+        <v>164</v>
       </c>
       <c r="H165" s="5" t="n">
         <v>1</v>
@@ -3730,17 +3739,17 @@
     </row>
     <row r="166" ht="25" customHeight="true">
       <c r="A166" s="4" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B166" s="4" t="e"/>
       <c r="C166" s="4" t="e"/>
       <c r="D166" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E166" s="4" t="e"/>
       <c r="F166" s="4" t="e"/>
       <c r="G166" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H166" s="5" t="n">
         <v>1</v>
@@ -3748,38 +3757,92 @@
     </row>
     <row r="167" ht="25" customHeight="true">
       <c r="A167" s="4" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B167" s="4" t="e"/>
       <c r="C167" s="4" t="e"/>
       <c r="D167" s="4" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E167" s="4" t="e"/>
       <c r="F167" s="4" t="e"/>
       <c r="G167" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H167" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="168" ht="25" customHeight="true">
+      <c r="A168" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="B168" s="4" t="e"/>
+      <c r="C168" s="4" t="e"/>
+      <c r="D168" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="E168" s="4" t="e"/>
+      <c r="F168" s="4" t="e"/>
+      <c r="G168" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="H168" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="169" ht="25" customHeight="true">
+      <c r="A169" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B169" s="4" t="e"/>
+      <c r="C169" s="4" t="e"/>
+      <c r="D169" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="E169" s="4" t="e"/>
+      <c r="F169" s="4" t="e"/>
+      <c r="G169" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H169" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="170" ht="25" customHeight="true">
+      <c r="A170" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="B170" s="4" t="e"/>
+      <c r="C170" s="4" t="e"/>
+      <c r="D170" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="E170" s="4" t="e"/>
+      <c r="F170" s="4" t="e"/>
+      <c r="G170" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="H167" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="168" ht="13" customHeight="true">
-      <c r="A168" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="B168" s="6" t="e"/>
-      <c r="C168" s="6" t="e"/>
-      <c r="D168" s="6" t="e"/>
-      <c r="E168" s="6" t="e"/>
-      <c r="F168" s="6" t="e"/>
-      <c r="G168" s="6" t="e"/>
-      <c r="H168" s="7" t="n">
-        <v>162</v>
+      <c r="H170" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171" ht="13" customHeight="true">
+      <c r="A171" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="B171" s="6" t="e"/>
+      <c r="C171" s="6" t="e"/>
+      <c r="D171" s="6" t="e"/>
+      <c r="E171" s="6" t="e"/>
+      <c r="F171" s="6" t="e"/>
+      <c r="G171" s="6" t="e"/>
+      <c r="H171" s="7" t="n">
+        <v>165</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="321">
+  <mergeCells count="327">
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="D8:F8"/>
     <mergeCell ref="A9:C9"/>
@@ -4100,7 +4163,13 @@
     <mergeCell ref="D166:F166"/>
     <mergeCell ref="A167:C167"/>
     <mergeCell ref="D167:F167"/>
-    <mergeCell ref="A168:G168"/>
+    <mergeCell ref="A168:C168"/>
+    <mergeCell ref="D168:F168"/>
+    <mergeCell ref="A169:C169"/>
+    <mergeCell ref="D169:F169"/>
+    <mergeCell ref="A170:C170"/>
+    <mergeCell ref="D170:F170"/>
+    <mergeCell ref="A171:G171"/>
   </mergeCells>
   <pageMargins left="0.393700787401574803149606299" top="0.393700787401574803149606299" right="0.393700787401574803149606299" bottom="0.393700787401574803149606299" header="0" footer="0"/>
   <pageSetup blackAndWhite="false" fitToHeight="0" fitToWidth="1" pageOrder="overThenDown" orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
Add new VTB accounts for ИП Маневич and ООО Реактив in accounts.json; update company account lists in companies.json accordingly.
</commit_message>
<xml_diff>
--- a/Расчетные счета.xlsx
+++ b/Расчетные счета.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="224">
   <si>
     <t>Параметры:</t>
   </si>
@@ -466,6 +466,9 @@
     <t>ООО "Реактив"</t>
   </si>
   <si>
+    <t>40702810400810170658</t>
+  </si>
+  <si>
     <t>40702810555000133589</t>
   </si>
   <si>
@@ -506,6 +509,9 @@
   </si>
   <si>
     <t>ООО "СЕВЕРНАЯ ЗВЕЗДА"</t>
+  </si>
+  <si>
+    <t>40702810900810159865</t>
   </si>
   <si>
     <t>40702810955710006991</t>
@@ -844,7 +850,7 @@
     <outlinePr summaryBelow="false" summaryRight="false"/>
     <pageSetUpPr autoPageBreaks="false" fitToPage="true"/>
   </sheetPr>
-  <dimension ref="H171"/>
+  <dimension ref="H173"/>
   <sheetFormatPr defaultColWidth="10.5" customHeight="true" defaultRowHeight="11.429"/>
   <cols>
     <col min="1" max="1" width="10.5" style="1" customWidth="true"/>
@@ -962,7 +968,7 @@
         <v>15</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" ht="25" customHeight="true">
@@ -2849,7 +2855,7 @@
       <c r="E116" s="4" t="e"/>
       <c r="F116" s="4" t="e"/>
       <c r="G116" s="4" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H116" s="5" t="n">
         <v>1</v>
@@ -2867,7 +2873,7 @@
       <c r="E117" s="4" t="e"/>
       <c r="F117" s="4" t="e"/>
       <c r="G117" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="H117" s="5" t="n">
         <v>1</v>
@@ -2898,12 +2904,12 @@
       <c r="B119" s="4" t="e"/>
       <c r="C119" s="4" t="e"/>
       <c r="D119" s="4" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="E119" s="4" t="e"/>
       <c r="F119" s="4" t="e"/>
       <c r="G119" s="4" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="H119" s="5" t="n">
         <v>1</v>
@@ -2911,12 +2917,12 @@
     </row>
     <row r="120" ht="25" customHeight="true">
       <c r="A120" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B120" s="4" t="e"/>
       <c r="C120" s="4" t="e"/>
       <c r="D120" s="4" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E120" s="4" t="e"/>
       <c r="F120" s="4" t="e"/>
@@ -2934,12 +2940,12 @@
       <c r="B121" s="4" t="e"/>
       <c r="C121" s="4" t="e"/>
       <c r="D121" s="4" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E121" s="4" t="e"/>
       <c r="F121" s="4" t="e"/>
       <c r="G121" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H121" s="5" t="n">
         <v>1</v>
@@ -2952,12 +2958,12 @@
       <c r="B122" s="4" t="e"/>
       <c r="C122" s="4" t="e"/>
       <c r="D122" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E122" s="4" t="e"/>
       <c r="F122" s="4" t="e"/>
       <c r="G122" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H122" s="5" t="n">
         <v>1</v>
@@ -2965,17 +2971,17 @@
     </row>
     <row r="123" ht="25" customHeight="true">
       <c r="A123" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B123" s="4" t="e"/>
       <c r="C123" s="4" t="e"/>
       <c r="D123" s="4" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E123" s="4" t="e"/>
       <c r="F123" s="4" t="e"/>
       <c r="G123" s="4" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H123" s="5" t="n">
         <v>1</v>
@@ -2988,12 +2994,12 @@
       <c r="B124" s="4" t="e"/>
       <c r="C124" s="4" t="e"/>
       <c r="D124" s="4" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E124" s="4" t="e"/>
       <c r="F124" s="4" t="e"/>
       <c r="G124" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H124" s="5" t="n">
         <v>1</v>
@@ -3006,12 +3012,12 @@
       <c r="B125" s="4" t="e"/>
       <c r="C125" s="4" t="e"/>
       <c r="D125" s="4" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E125" s="4" t="e"/>
       <c r="F125" s="4" t="e"/>
       <c r="G125" s="4" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="H125" s="5" t="n">
         <v>1</v>
@@ -3024,33 +3030,33 @@
       <c r="B126" s="4" t="e"/>
       <c r="C126" s="4" t="e"/>
       <c r="D126" s="4" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="E126" s="4" t="e"/>
       <c r="F126" s="4" t="e"/>
       <c r="G126" s="4" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="H126" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="127" ht="25" customHeight="true">
       <c r="A127" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B127" s="4" t="e"/>
       <c r="C127" s="4" t="e"/>
       <c r="D127" s="4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E127" s="4" t="e"/>
       <c r="F127" s="4" t="e"/>
       <c r="G127" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H127" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="128" ht="25" customHeight="true">
@@ -3060,12 +3066,12 @@
       <c r="B128" s="4" t="e"/>
       <c r="C128" s="4" t="e"/>
       <c r="D128" s="4" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E128" s="4" t="e"/>
       <c r="F128" s="4" t="e"/>
       <c r="G128" s="4" t="s">
-        <v>164</v>
+        <v>15</v>
       </c>
       <c r="H128" s="5" t="n">
         <v>1</v>
@@ -3073,17 +3079,17 @@
     </row>
     <row r="129" ht="25" customHeight="true">
       <c r="A129" s="4" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B129" s="4" t="e"/>
       <c r="C129" s="4" t="e"/>
       <c r="D129" s="4" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="E129" s="4" t="e"/>
       <c r="F129" s="4" t="e"/>
       <c r="G129" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H129" s="5" t="n">
         <v>1</v>
@@ -3091,17 +3097,17 @@
     </row>
     <row r="130" ht="25" customHeight="true">
       <c r="A130" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B130" s="4" t="e"/>
       <c r="C130" s="4" t="e"/>
       <c r="D130" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E130" s="4" t="e"/>
       <c r="F130" s="4" t="e"/>
       <c r="G130" s="4" t="s">
-        <v>11</v>
+        <v>166</v>
       </c>
       <c r="H130" s="5" t="n">
         <v>1</v>
@@ -3109,17 +3115,17 @@
     </row>
     <row r="131" ht="25" customHeight="true">
       <c r="A131" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B131" s="4" t="e"/>
       <c r="C131" s="4" t="e"/>
       <c r="D131" s="4" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="E131" s="4" t="e"/>
       <c r="F131" s="4" t="e"/>
       <c r="G131" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H131" s="5" t="n">
         <v>1</v>
@@ -3132,12 +3138,12 @@
       <c r="B132" s="4" t="e"/>
       <c r="C132" s="4" t="e"/>
       <c r="D132" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E132" s="4" t="e"/>
       <c r="F132" s="4" t="e"/>
       <c r="G132" s="4" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="H132" s="5" t="n">
         <v>1</v>
@@ -3145,17 +3151,17 @@
     </row>
     <row r="133" ht="25" customHeight="true">
       <c r="A133" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B133" s="4" t="e"/>
       <c r="C133" s="4" t="e"/>
       <c r="D133" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E133" s="4" t="e"/>
       <c r="F133" s="4" t="e"/>
       <c r="G133" s="4" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H133" s="5" t="n">
         <v>1</v>
@@ -3163,17 +3169,17 @@
     </row>
     <row r="134" ht="25" customHeight="true">
       <c r="A134" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B134" s="4" t="e"/>
       <c r="C134" s="4" t="e"/>
       <c r="D134" s="4" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E134" s="4" t="e"/>
       <c r="F134" s="4" t="e"/>
       <c r="G134" s="4" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="H134" s="5" t="n">
         <v>1</v>
@@ -3186,12 +3192,12 @@
       <c r="B135" s="4" t="e"/>
       <c r="C135" s="4" t="e"/>
       <c r="D135" s="4" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E135" s="4" t="e"/>
       <c r="F135" s="4" t="e"/>
       <c r="G135" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="H135" s="5" t="n">
         <v>1</v>
@@ -3204,7 +3210,7 @@
       <c r="B136" s="4" t="e"/>
       <c r="C136" s="4" t="e"/>
       <c r="D136" s="4" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E136" s="4" t="e"/>
       <c r="F136" s="4" t="e"/>
@@ -3222,7 +3228,7 @@
       <c r="B137" s="4" t="e"/>
       <c r="C137" s="4" t="e"/>
       <c r="D137" s="4" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E137" s="4" t="e"/>
       <c r="F137" s="4" t="e"/>
@@ -3240,7 +3246,7 @@
       <c r="B138" s="4" t="e"/>
       <c r="C138" s="4" t="e"/>
       <c r="D138" s="4" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E138" s="4" t="e"/>
       <c r="F138" s="4" t="e"/>
@@ -3258,7 +3264,7 @@
       <c r="B139" s="4" t="e"/>
       <c r="C139" s="4" t="e"/>
       <c r="D139" s="4" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E139" s="4" t="e"/>
       <c r="F139" s="4" t="e"/>
@@ -3276,7 +3282,7 @@
       <c r="B140" s="4" t="e"/>
       <c r="C140" s="4" t="e"/>
       <c r="D140" s="4" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E140" s="4" t="e"/>
       <c r="F140" s="4" t="e"/>
@@ -3294,12 +3300,12 @@
       <c r="B141" s="4" t="e"/>
       <c r="C141" s="4" t="e"/>
       <c r="D141" s="4" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="E141" s="4" t="e"/>
       <c r="F141" s="4" t="e"/>
       <c r="G141" s="4" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="H141" s="5" t="n">
         <v>1</v>
@@ -3307,17 +3313,17 @@
     </row>
     <row r="142" ht="25" customHeight="true">
       <c r="A142" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B142" s="4" t="e"/>
       <c r="C142" s="4" t="e"/>
       <c r="D142" s="4" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="E142" s="4" t="e"/>
       <c r="F142" s="4" t="e"/>
       <c r="G142" s="4" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="H142" s="5" t="n">
         <v>1</v>
@@ -3325,12 +3331,12 @@
     </row>
     <row r="143" ht="25" customHeight="true">
       <c r="A143" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B143" s="4" t="e"/>
       <c r="C143" s="4" t="e"/>
       <c r="D143" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E143" s="4" t="e"/>
       <c r="F143" s="4" t="e"/>
@@ -3343,12 +3349,12 @@
     </row>
     <row r="144" ht="25" customHeight="true">
       <c r="A144" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B144" s="4" t="e"/>
       <c r="C144" s="4" t="e"/>
       <c r="D144" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E144" s="4" t="e"/>
       <c r="F144" s="4" t="e"/>
@@ -3361,17 +3367,17 @@
     </row>
     <row r="145" ht="25" customHeight="true">
       <c r="A145" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B145" s="4" t="e"/>
       <c r="C145" s="4" t="e"/>
       <c r="D145" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E145" s="4" t="e"/>
       <c r="F145" s="4" t="e"/>
       <c r="G145" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H145" s="5" t="n">
         <v>1</v>
@@ -3379,17 +3385,17 @@
     </row>
     <row r="146" ht="25" customHeight="true">
       <c r="A146" s="4" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B146" s="4" t="e"/>
       <c r="C146" s="4" t="e"/>
       <c r="D146" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E146" s="4" t="e"/>
       <c r="F146" s="4" t="e"/>
       <c r="G146" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H146" s="5" t="n">
         <v>1</v>
@@ -3397,17 +3403,17 @@
     </row>
     <row r="147" ht="25" customHeight="true">
       <c r="A147" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B147" s="4" t="e"/>
       <c r="C147" s="4" t="e"/>
       <c r="D147" s="4" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E147" s="4" t="e"/>
       <c r="F147" s="4" t="e"/>
       <c r="G147" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H147" s="5" t="n">
         <v>1</v>
@@ -3420,12 +3426,12 @@
       <c r="B148" s="4" t="e"/>
       <c r="C148" s="4" t="e"/>
       <c r="D148" s="4" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E148" s="4" t="e"/>
       <c r="F148" s="4" t="e"/>
       <c r="G148" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H148" s="5" t="n">
         <v>1</v>
@@ -3438,12 +3444,12 @@
       <c r="B149" s="4" t="e"/>
       <c r="C149" s="4" t="e"/>
       <c r="D149" s="4" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="E149" s="4" t="e"/>
       <c r="F149" s="4" t="e"/>
       <c r="G149" s="4" t="s">
-        <v>164</v>
+        <v>15</v>
       </c>
       <c r="H149" s="5" t="n">
         <v>1</v>
@@ -3451,17 +3457,17 @@
     </row>
     <row r="150" ht="25" customHeight="true">
       <c r="A150" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B150" s="4" t="e"/>
       <c r="C150" s="4" t="e"/>
       <c r="D150" s="4" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="E150" s="4" t="e"/>
       <c r="F150" s="4" t="e"/>
       <c r="G150" s="4" t="s">
-        <v>164</v>
+        <v>13</v>
       </c>
       <c r="H150" s="5" t="n">
         <v>1</v>
@@ -3469,17 +3475,17 @@
     </row>
     <row r="151" ht="25" customHeight="true">
       <c r="A151" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B151" s="4" t="e"/>
       <c r="C151" s="4" t="e"/>
       <c r="D151" s="4" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E151" s="4" t="e"/>
       <c r="F151" s="4" t="e"/>
       <c r="G151" s="4" t="s">
-        <v>13</v>
+        <v>166</v>
       </c>
       <c r="H151" s="5" t="n">
         <v>1</v>
@@ -3487,7 +3493,7 @@
     </row>
     <row r="152" ht="25" customHeight="true">
       <c r="A152" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B152" s="4" t="e"/>
       <c r="C152" s="4" t="e"/>
@@ -3497,7 +3503,7 @@
       <c r="E152" s="4" t="e"/>
       <c r="F152" s="4" t="e"/>
       <c r="G152" s="4" t="s">
-        <v>11</v>
+        <v>166</v>
       </c>
       <c r="H152" s="5" t="n">
         <v>1</v>
@@ -3505,17 +3511,17 @@
     </row>
     <row r="153" ht="25" customHeight="true">
       <c r="A153" s="4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B153" s="4" t="e"/>
       <c r="C153" s="4" t="e"/>
       <c r="D153" s="4" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E153" s="4" t="e"/>
       <c r="F153" s="4" t="e"/>
       <c r="G153" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H153" s="5" t="n">
         <v>1</v>
@@ -3528,12 +3534,12 @@
       <c r="B154" s="4" t="e"/>
       <c r="C154" s="4" t="e"/>
       <c r="D154" s="4" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E154" s="4" t="e"/>
       <c r="F154" s="4" t="e"/>
       <c r="G154" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H154" s="5" t="n">
         <v>1</v>
@@ -3546,12 +3552,12 @@
       <c r="B155" s="4" t="e"/>
       <c r="C155" s="4" t="e"/>
       <c r="D155" s="4" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E155" s="4" t="e"/>
       <c r="F155" s="4" t="e"/>
       <c r="G155" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H155" s="5" t="n">
         <v>1</v>
@@ -3564,7 +3570,7 @@
       <c r="B156" s="4" t="e"/>
       <c r="C156" s="4" t="e"/>
       <c r="D156" s="4" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E156" s="4" t="e"/>
       <c r="F156" s="4" t="e"/>
@@ -3582,7 +3588,7 @@
       <c r="B157" s="4" t="e"/>
       <c r="C157" s="4" t="e"/>
       <c r="D157" s="4" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E157" s="4" t="e"/>
       <c r="F157" s="4" t="e"/>
@@ -3600,7 +3606,7 @@
       <c r="B158" s="4" t="e"/>
       <c r="C158" s="4" t="e"/>
       <c r="D158" s="4" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E158" s="4" t="e"/>
       <c r="F158" s="4" t="e"/>
@@ -3618,7 +3624,7 @@
       <c r="B159" s="4" t="e"/>
       <c r="C159" s="4" t="e"/>
       <c r="D159" s="4" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E159" s="4" t="e"/>
       <c r="F159" s="4" t="e"/>
@@ -3636,7 +3642,7 @@
       <c r="B160" s="4" t="e"/>
       <c r="C160" s="4" t="e"/>
       <c r="D160" s="4" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E160" s="4" t="e"/>
       <c r="F160" s="4" t="e"/>
@@ -3654,7 +3660,7 @@
       <c r="B161" s="4" t="e"/>
       <c r="C161" s="4" t="e"/>
       <c r="D161" s="4" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="E161" s="4" t="e"/>
       <c r="F161" s="4" t="e"/>
@@ -3667,17 +3673,17 @@
     </row>
     <row r="162" ht="25" customHeight="true">
       <c r="A162" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B162" s="4" t="e"/>
       <c r="C162" s="4" t="e"/>
       <c r="D162" s="4" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="E162" s="4" t="e"/>
       <c r="F162" s="4" t="e"/>
       <c r="G162" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H162" s="5" t="n">
         <v>1</v>
@@ -3685,12 +3691,12 @@
     </row>
     <row r="163" ht="25" customHeight="true">
       <c r="A163" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B163" s="4" t="e"/>
       <c r="C163" s="4" t="e"/>
       <c r="D163" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E163" s="4" t="e"/>
       <c r="F163" s="4" t="e"/>
@@ -3703,12 +3709,12 @@
     </row>
     <row r="164" ht="25" customHeight="true">
       <c r="A164" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B164" s="4" t="e"/>
       <c r="C164" s="4" t="e"/>
       <c r="D164" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E164" s="4" t="e"/>
       <c r="F164" s="4" t="e"/>
@@ -3721,17 +3727,17 @@
     </row>
     <row r="165" ht="25" customHeight="true">
       <c r="A165" s="4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B165" s="4" t="e"/>
       <c r="C165" s="4" t="e"/>
       <c r="D165" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E165" s="4" t="e"/>
       <c r="F165" s="4" t="e"/>
       <c r="G165" s="4" t="s">
-        <v>164</v>
+        <v>13</v>
       </c>
       <c r="H165" s="5" t="n">
         <v>1</v>
@@ -3739,17 +3745,17 @@
     </row>
     <row r="166" ht="25" customHeight="true">
       <c r="A166" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B166" s="4" t="e"/>
       <c r="C166" s="4" t="e"/>
       <c r="D166" s="4" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="E166" s="4" t="e"/>
       <c r="F166" s="4" t="e"/>
       <c r="G166" s="4" t="s">
-        <v>59</v>
+        <v>11</v>
       </c>
       <c r="H166" s="5" t="n">
         <v>1</v>
@@ -3757,17 +3763,17 @@
     </row>
     <row r="167" ht="25" customHeight="true">
       <c r="A167" s="4" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B167" s="4" t="e"/>
       <c r="C167" s="4" t="e"/>
       <c r="D167" s="4" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="E167" s="4" t="e"/>
       <c r="F167" s="4" t="e"/>
       <c r="G167" s="4" t="s">
-        <v>59</v>
+        <v>166</v>
       </c>
       <c r="H167" s="5" t="n">
         <v>1</v>
@@ -3775,17 +3781,17 @@
     </row>
     <row r="168" ht="25" customHeight="true">
       <c r="A168" s="4" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B168" s="4" t="e"/>
       <c r="C168" s="4" t="e"/>
       <c r="D168" s="4" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="E168" s="4" t="e"/>
       <c r="F168" s="4" t="e"/>
       <c r="G168" s="4" t="s">
-        <v>219</v>
+        <v>59</v>
       </c>
       <c r="H168" s="5" t="n">
         <v>1</v>
@@ -3793,7 +3799,7 @@
     </row>
     <row r="169" ht="25" customHeight="true">
       <c r="A169" s="4" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B169" s="4" t="e"/>
       <c r="C169" s="4" t="e"/>
@@ -3811,38 +3817,74 @@
     </row>
     <row r="170" ht="25" customHeight="true">
       <c r="A170" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B170" s="4" t="e"/>
       <c r="C170" s="4" t="e"/>
       <c r="D170" s="4" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="E170" s="4" t="e"/>
       <c r="F170" s="4" t="e"/>
       <c r="G170" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="H170" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171" ht="25" customHeight="true">
+      <c r="A171" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="B171" s="4" t="e"/>
+      <c r="C171" s="4" t="e"/>
+      <c r="D171" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="E171" s="4" t="e"/>
+      <c r="F171" s="4" t="e"/>
+      <c r="G171" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H171" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="172" ht="25" customHeight="true">
+      <c r="A172" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="B172" s="4" t="e"/>
+      <c r="C172" s="4" t="e"/>
+      <c r="D172" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="E172" s="4" t="e"/>
+      <c r="F172" s="4" t="e"/>
+      <c r="G172" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="H170" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="171" ht="13" customHeight="true">
-      <c r="A171" s="6" t="s">
-        <v>221</v>
-      </c>
-      <c r="B171" s="6" t="e"/>
-      <c r="C171" s="6" t="e"/>
-      <c r="D171" s="6" t="e"/>
-      <c r="E171" s="6" t="e"/>
-      <c r="F171" s="6" t="e"/>
-      <c r="G171" s="6" t="e"/>
-      <c r="H171" s="7" t="n">
-        <v>165</v>
+      <c r="H172" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="173" ht="13" customHeight="true">
+      <c r="A173" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="B173" s="6" t="e"/>
+      <c r="C173" s="6" t="e"/>
+      <c r="D173" s="6" t="e"/>
+      <c r="E173" s="6" t="e"/>
+      <c r="F173" s="6" t="e"/>
+      <c r="G173" s="6" t="e"/>
+      <c r="H173" s="7" t="n">
+        <v>168</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="327">
+  <mergeCells count="331">
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="D8:F8"/>
     <mergeCell ref="A9:C9"/>
@@ -4169,7 +4211,11 @@
     <mergeCell ref="D169:F169"/>
     <mergeCell ref="A170:C170"/>
     <mergeCell ref="D170:F170"/>
-    <mergeCell ref="A171:G171"/>
+    <mergeCell ref="A171:C171"/>
+    <mergeCell ref="D171:F171"/>
+    <mergeCell ref="A172:C172"/>
+    <mergeCell ref="D172:F172"/>
+    <mergeCell ref="A173:G173"/>
   </mergeCells>
   <pageMargins left="0.393700787401574803149606299" top="0.393700787401574803149606299" right="0.393700787401574803149606299" bottom="0.393700787401574803149606299" header="0" footer="0"/>
   <pageSetup blackAndWhite="false" fitToHeight="0" fitToWidth="1" pageOrder="overThenDown" orientation="portrait" paperSize="9"/>

</xml_diff>